<commit_message>
CI template: Instructor Name on Sheet 2 is now a dropdown from Sheet 1
Column A of Course Appointments sheet now validates against the
InstructorList named range (Instructors!$A$2:$A$51), so users pick
from whoever was entered on the Instructors tab instead of retyping
the name — eliminates mismatch errors on import.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nlh-platform/public/CI_Import_Template.xlsx
+++ b/nlh-platform/public/CI_Import_Template.xlsx
@@ -29,6 +29,7 @@
     <definedName name="Rubiks_Cube">Lists!$O$2:$O$3</definedName>
     <definedName name="Storytelling">Lists!$P$2:$P$4</definedName>
     <definedName name="Write_Well">Lists!$Q$2:$Q$6</definedName>
+    <definedName name="InstructorList">Instructors!$A$2:$A$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +55,9 @@
     <font>
       <name val="DM Sans"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -79,30 +83,26 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00CCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00CCCCCC"/>
       </right>
-      <top style="thin">
-        <color rgb="00DDDDDD"/>
-      </top>
       <bottom style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -177,6 +177,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>NLH Platform</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>Select from the list — names come from the Instructors sheet tab</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -468,18 +483,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -639,9 +654,449 @@
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="n"/>
+      <c r="I44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+      <c r="I46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="n"/>
+      <c r="I47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
+      <c r="H49" s="2" t="n"/>
+      <c r="I49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="n"/>
+      <c r="H50" s="2" t="n"/>
+      <c r="I50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="2" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
       <formula1>"active,inactive"</formula1>
     </dataValidation>
   </dataValidations>
@@ -655,13 +1110,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
@@ -778,9 +1233,332 @@
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+    </row>
   </sheetData>
-  <dataValidations count="53">
-    <dataValidation sqref="B2:B51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="54">
+    <dataValidation sqref="A2:A51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
+      <formula1>InstructorList</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
       <formula1>CourseList</formula1>
     </dataValidation>
     <dataValidation sqref="C2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -933,14 +1711,15 @@
     <dataValidation sqref="C51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=INDIRECT(SUBSTITUTE(B51," ","_"))</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
       <formula1>"per_session,per_student,monthly"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -954,9 +1733,89 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Course</t>
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>CourseList</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>ACEM_Abacus</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Art_and_Craft</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Chess</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Coding</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Computer</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Creative_Writing</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Easy_Math</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>English_Grammar</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Montessori</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Personality_Dev</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Phonics</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Public_Speaking</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Rubiks_Cube</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>Storytelling</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>Write_Well</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix CI template: instructor dropdown now reliably mirrors Sheet 1 names
The cross-sheet named range (Instructors!A2:A51) wasn't resolving in
Excel's data validation. Fix: Lists sheet now has a mirror column with
=IF(Instructors!Ax="","",Instructors!Ax) formulas; InstructorList named
range points to that same-sheet column (Lists!R2:R51) which Excel
always resolves correctly in dropdowns.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nlh-platform/public/CI_Import_Template.xlsx
+++ b/nlh-platform/public/CI_Import_Template.xlsx
@@ -29,7 +29,7 @@
     <definedName name="Rubiks_Cube">Lists!$O$2:$O$3</definedName>
     <definedName name="Storytelling">Lists!$P$2:$P$4</definedName>
     <definedName name="Write_Well">Lists!$Q$2:$Q$6</definedName>
-    <definedName name="InstructorList">Instructors!$A$2:$A$51</definedName>
+    <definedName name="InstructorList">Lists!$R$2:$R$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -47,20 +47,20 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="DM Sans"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="DM Sans"/>
+      <name val="Arial"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -72,25 +72,19 @@
         <fgColor rgb="00534AB7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAE8F7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -101,7 +95,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -177,21 +173,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>NLH Platform</author>
-  </authors>
-  <commentList>
-    <comment ref="A2" authorId="0" shapeId="0">
-      <text>
-        <t>Select from the list — names come from the Instructors sheet tab</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -483,16 +464,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
@@ -525,7 +506,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Area / Locality</t>
+          <t>Area/Locality</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -654,449 +635,9 @@
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-      <c r="G41" s="2" t="n"/>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-      <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
-      <c r="G46" s="2" t="n"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="2" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
-      <c r="G49" s="2" t="n"/>
-      <c r="H49" s="2" t="n"/>
-      <c r="I49" s="2" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="n"/>
-      <c r="G50" s="2" t="n"/>
-      <c r="H50" s="2" t="n"/>
-      <c r="I50" s="2" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="2" t="n"/>
-      <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="n"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
+    <dataValidation sqref="I2:I51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"active,inactive"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1110,14 +651,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1233,332 +774,12 @@
       <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="n"/>
-    </row>
   </sheetData>
   <dataValidations count="54">
-    <dataValidation sqref="A2:A51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
+    <dataValidation sqref="A2:A51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>InstructorList</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
+    <dataValidation sqref="B2:B51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>CourseList</formula1>
     </dataValidation>
     <dataValidation sqref="C2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1711,15 +932,14 @@
     <dataValidation sqref="C51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=INDIRECT(SUBSTITUTE(B51," ","_"))</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
+    <dataValidation sqref="D2:D51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"per_session,per_student,monthly"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F51" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please choose a value from the dropdown list." type="list">
+    <dataValidation sqref="F2:F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1729,93 +949,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>CourseList</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>ACEM_Abacus</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Art_and_Craft</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Chess</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Coding</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Computer</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Creative_Writing</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Easy_Math</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>English_Grammar</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
-        <is>
-          <t>Montessori</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>Personality_Dev</t>
-        </is>
-      </c>
-      <c r="L1" s="3" t="inlineStr">
-        <is>
-          <t>Phonics</t>
-        </is>
-      </c>
-      <c r="M1" s="3" t="inlineStr">
-        <is>
-          <t>Public_Speaking</t>
-        </is>
-      </c>
-      <c r="N1" s="3" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="O1" s="3" t="inlineStr">
-        <is>
-          <t>Rubiks_Cube</t>
-        </is>
-      </c>
-      <c r="P1" s="3" t="inlineStr">
-        <is>
-          <t>Storytelling</t>
-        </is>
-      </c>
-      <c r="Q1" s="3" t="inlineStr">
-        <is>
-          <t>Write_Well</t>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>InstructorNames</t>
         </is>
       </c>
     </row>
@@ -1905,6 +1050,10 @@
           <t>Print HW</t>
         </is>
       </c>
+      <c r="R2">
+        <f>IF(Instructors!A2="","",Instructors!A2)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1982,6 +1131,10 @@
           <t>English HW Junior</t>
         </is>
       </c>
+      <c r="R3">
+        <f>IF(Instructors!A3="","",Instructors!A3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2049,6 +1202,10 @@
           <t>English HW Senior</t>
         </is>
       </c>
+      <c r="R4">
+        <f>IF(Instructors!A4="","",Instructors!A4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2076,6 +1233,10 @@
           <t>Hindi HW</t>
         </is>
       </c>
+      <c r="R5">
+        <f>IF(Instructors!A5="","",Instructors!A5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2098,6 +1259,10 @@
           <t>Calligraphy</t>
         </is>
       </c>
+      <c r="R6">
+        <f>IF(Instructors!A6="","",Instructors!A6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2110,6 +1275,10 @@
           <t>Jr Level 5</t>
         </is>
       </c>
+      <c r="R7">
+        <f>IF(Instructors!A7="","",Instructors!A7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2122,6 +1291,10 @@
           <t>Jr Level 6</t>
         </is>
       </c>
+      <c r="R8">
+        <f>IF(Instructors!A8="","",Instructors!A8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2134,6 +1307,10 @@
           <t>Sr Level 1</t>
         </is>
       </c>
+      <c r="R9">
+        <f>IF(Instructors!A9="","",Instructors!A9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2146,6 +1323,10 @@
           <t>Sr Level 2</t>
         </is>
       </c>
+      <c r="R10">
+        <f>IF(Instructors!A10="","",Instructors!A10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2158,6 +1339,10 @@
           <t>Sr Level 3</t>
         </is>
       </c>
+      <c r="R11">
+        <f>IF(Instructors!A11="","",Instructors!A11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2170,6 +1355,10 @@
           <t>Sr Level 4</t>
         </is>
       </c>
+      <c r="R12">
+        <f>IF(Instructors!A12="","",Instructors!A12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2182,6 +1371,10 @@
           <t>Sr Level 5</t>
         </is>
       </c>
+      <c r="R13">
+        <f>IF(Instructors!A13="","",Instructors!A13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2194,6 +1387,10 @@
           <t>Sr Level 6</t>
         </is>
       </c>
+      <c r="R14">
+        <f>IF(Instructors!A14="","",Instructors!A14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2201,6 +1398,10 @@
           <t>Rubiks Cube</t>
         </is>
       </c>
+      <c r="R15">
+        <f>IF(Instructors!A15="","",Instructors!A15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2208,12 +1409,224 @@
           <t>Storytelling</t>
         </is>
       </c>
+      <c r="R16">
+        <f>IF(Instructors!A16="","",Instructors!A16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
           <t>Write Well</t>
         </is>
+      </c>
+      <c r="R17">
+        <f>IF(Instructors!A17="","",Instructors!A17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="R18">
+        <f>IF(Instructors!A18="","",Instructors!A18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="R19">
+        <f>IF(Instructors!A19="","",Instructors!A19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="R20">
+        <f>IF(Instructors!A20="","",Instructors!A20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="R21">
+        <f>IF(Instructors!A21="","",Instructors!A21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="R22">
+        <f>IF(Instructors!A22="","",Instructors!A22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="R23">
+        <f>IF(Instructors!A23="","",Instructors!A23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="R24">
+        <f>IF(Instructors!A24="","",Instructors!A24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="R25">
+        <f>IF(Instructors!A25="","",Instructors!A25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="R26">
+        <f>IF(Instructors!A26="","",Instructors!A26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="R27">
+        <f>IF(Instructors!A27="","",Instructors!A27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="R28">
+        <f>IF(Instructors!A28="","",Instructors!A28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="R29">
+        <f>IF(Instructors!A29="","",Instructors!A29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="R30">
+        <f>IF(Instructors!A30="","",Instructors!A30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="R31">
+        <f>IF(Instructors!A31="","",Instructors!A31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="R32">
+        <f>IF(Instructors!A32="","",Instructors!A32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="R33">
+        <f>IF(Instructors!A33="","",Instructors!A33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="R34">
+        <f>IF(Instructors!A34="","",Instructors!A34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="R35">
+        <f>IF(Instructors!A35="","",Instructors!A35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="R36">
+        <f>IF(Instructors!A36="","",Instructors!A36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="R37">
+        <f>IF(Instructors!A37="","",Instructors!A37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="R38">
+        <f>IF(Instructors!A38="","",Instructors!A38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="R39">
+        <f>IF(Instructors!A39="","",Instructors!A39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="R40">
+        <f>IF(Instructors!A40="","",Instructors!A40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="R41">
+        <f>IF(Instructors!A41="","",Instructors!A41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="R42">
+        <f>IF(Instructors!A42="","",Instructors!A42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="R43">
+        <f>IF(Instructors!A43="","",Instructors!A43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="R44">
+        <f>IF(Instructors!A44="","",Instructors!A44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="R45">
+        <f>IF(Instructors!A45="","",Instructors!A45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="R46">
+        <f>IF(Instructors!A46="","",Instructors!A46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="R47">
+        <f>IF(Instructors!A47="","",Instructors!A47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="R48">
+        <f>IF(Instructors!A48="","",Instructors!A48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="R49">
+        <f>IF(Instructors!A49="","",Instructors!A49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="R50">
+        <f>IF(Instructors!A50="","",Instructors!A50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="R51">
+        <f>IF(Instructors!A51="","",Instructors!A51)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>